<commit_message>
Improve production tracking and dashboard proof records
</commit_message>
<xml_diff>
--- a/data/aruco_markers/aruco_marker_employee_assignment_with_images.xlsx
+++ b/data/aruco_markers/aruco_marker_employee_assignment_with_images.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gate.office\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://woodcorp1-my.sharepoint.com/personal/dheeraj_kumar_gumcorp_com/Documents/Desktop/Factory_Ai_System/data/aruco_markers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F132AB-8932-4AC1-9138-8661C4B318E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{52F132AB-8932-4AC1-9138-8661C4B318E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4FB27D4-F3A0-42AC-83A2-DDBE4E470079}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Marker Assignment" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="41">
   <si>
     <t>marker_id</t>
   </si>
@@ -130,9 +130,6 @@
     <t>Fida</t>
   </si>
   <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>Zaid Ali 1</t>
   </si>
   <si>
@@ -143,6 +140,9 @@
   </si>
   <si>
     <t>Cleaner</t>
+  </si>
+  <si>
+    <t>Mamtaz</t>
   </si>
 </sst>
 </file>
@@ -867,6 +867,44 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>190500</xdr:colOff>
       <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>942975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="marker_17_Employee_17.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -877,17 +915,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="marker_17_Employee_17.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <xdr:cNvPr id="20" name="marker_18_Employee_18.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -915,17 +953,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="20" name="marker_18_Employee_18.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <xdr:cNvPr id="21" name="marker_19_Employee_19.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -953,17 +991,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="marker_19_Employee_19.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <xdr:cNvPr id="22" name="marker_20_Employee_20.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -991,17 +1029,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="marker_20_Employee_20.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <xdr:cNvPr id="23" name="marker_21_Employee_21.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1029,17 +1067,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="marker_21_Employee_21.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <xdr:cNvPr id="24" name="marker_22_Employee_22.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1067,17 +1105,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="24" name="marker_22_Employee_22.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <xdr:cNvPr id="25" name="marker_23_Employee_23.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1105,17 +1143,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="marker_23_Employee_23.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <xdr:cNvPr id="26" name="marker_24_Employee_24.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1143,17 +1181,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="marker_24_Employee_24.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <xdr:cNvPr id="27" name="marker_25_Employee_25.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1181,17 +1219,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="marker_25_Employee_25.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001B000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <xdr:cNvPr id="28" name="marker_26_Employee_26.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1219,17 +1257,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="28" name="marker_26_Employee_26.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001C000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <xdr:cNvPr id="29" name="marker_27_Employee_27.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1257,17 +1295,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="29" name="marker_27_Employee_27.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001D000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <xdr:cNvPr id="30" name="marker_28_Employee_28.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1295,17 +1333,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="30" name="marker_28_Employee_28.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <xdr:cNvPr id="31" name="marker_29_Employee_29.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1333,17 +1371,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="31" name="marker_29_Employee_29.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001F000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <xdr:cNvPr id="32" name="marker_30_Employee_30.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000020000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1371,17 +1409,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="32" name="marker_30_Employee_30.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000020000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
+        <xdr:cNvPr id="33" name="marker_31_Employee_31.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000021000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1409,17 +1447,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="33" name="marker_31_Employee_31.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000021000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
+        <xdr:cNvPr id="34" name="marker_32_Employee_32.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000022000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1447,17 +1485,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="34" name="marker_32_Employee_32.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000022000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33"/>
+        <xdr:cNvPr id="35" name="marker_33_Employee_33.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000023000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1485,17 +1523,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="35" name="marker_33_Employee_33.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000023000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34"/>
+        <xdr:cNvPr id="36" name="marker_34_Employee_34.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000024000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1523,17 +1561,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="36" name="marker_34_Employee_34.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000024000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
+        <xdr:cNvPr id="37" name="marker_35_Employee_35.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000025000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1551,6 +1589,82 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>190500</xdr:colOff>
       <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>942975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="marker_36_Employee_36.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000026000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>942975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="marker_37_Employee_37.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000027000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -1561,17 +1675,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="37" name="marker_35_Employee_35.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000025000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
+        <xdr:cNvPr id="40" name="marker_38_Employee_38.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000028000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1599,17 +1713,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="38" name="marker_36_Employee_36.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000026000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
+        <xdr:cNvPr id="41" name="marker_39_Employee_39.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000029000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1637,17 +1751,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="39" name="marker_37_Employee_37.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000027000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
+        <xdr:cNvPr id="42" name="marker_40_Employee_40.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1675,17 +1789,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="40" name="marker_38_Employee_38.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000028000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39"/>
+        <xdr:cNvPr id="43" name="marker_41_Employee_41.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1713,17 +1827,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="marker_39_Employee_39.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000029000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40"/>
+        <xdr:cNvPr id="44" name="marker_42_Employee_42.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1751,17 +1865,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="42" name="marker_40_Employee_40.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41"/>
+        <xdr:cNvPr id="45" name="marker_43_Employee_43.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1789,17 +1903,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="43" name="marker_41_Employee_41.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002B000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42"/>
+        <xdr:cNvPr id="46" name="marker_44_Employee_44.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1827,17 +1941,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="44" name="marker_42_Employee_42.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002C000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43"/>
+        <xdr:cNvPr id="47" name="marker_45_Employee_45.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1865,17 +1979,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="45" name="marker_43_Employee_43.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002D000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44"/>
+        <xdr:cNvPr id="48" name="marker_46_Employee_46.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000030000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1903,17 +2017,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="46" name="marker_44_Employee_44.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45"/>
+        <xdr:cNvPr id="49" name="marker_47_Employee_47.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000031000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1941,17 +2055,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="47" name="marker_45_Employee_45.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002F000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46"/>
+        <xdr:cNvPr id="50" name="marker_48_Employee_48.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000032000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1979,120 +2093,6 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="48" name="marker_46_Employee_46.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000030000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1190625</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="49" name="marker_47_Employee_47.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000031000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1190625</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="50" name="marker_48_Employee_48.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000032000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1190625</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
         <xdr:cNvPr id="51" name="marker_49_Employee_49.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
@@ -2109,6 +2109,48 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="marker_3_Usman.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{702E7B68-4B21-43E0-8527-FB4C3337AB9C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="857250" y="3514725"/>
+          <a:ext cx="1000125" cy="942975"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -2416,7 +2458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2466,8 +2508,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="81.95" customHeight="1">
-      <c r="A3" t="s">
-        <v>36</v>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>5</v>
@@ -2510,19 +2552,19 @@
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>5</v>
+        <v>40</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1284</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="81.95" customHeight="1">
@@ -2785,7 +2827,7 @@
     </row>
     <row r="19" spans="1:7" ht="81.95" customHeight="1">
       <c r="A19">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>5</v>
@@ -2805,7 +2847,7 @@
     </row>
     <row r="20" spans="1:7" ht="81.95" customHeight="1">
       <c r="A20">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>5</v>
@@ -2825,79 +2867,79 @@
     </row>
     <row r="21" spans="1:7" ht="81.95" customHeight="1">
       <c r="A21">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="81.95" customHeight="1">
       <c r="A22">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="81.95" customHeight="1">
       <c r="A23">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>5</v>
+        <v>38</v>
+      </c>
+      <c r="D23" s="2">
+        <v>1306</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="81.95" customHeight="1">
       <c r="A24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="2">
-        <v>1306</v>
+        <v>6</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>9</v>
@@ -2905,67 +2947,67 @@
     </row>
     <row r="25" spans="1:7" ht="81.95" customHeight="1">
       <c r="A25">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>7</v>
+        <v>33</v>
+      </c>
+      <c r="D25" s="2">
+        <v>1284</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="81.95" customHeight="1">
       <c r="A26">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D26" s="2">
-        <v>1284</v>
+        <v>36</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="81.95" customHeight="1">
       <c r="A27">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="81.95" customHeight="1">
       <c r="A28">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>5</v>
@@ -2985,7 +3027,7 @@
     </row>
     <row r="29" spans="1:7" ht="81.95" customHeight="1">
       <c r="A29">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>5</v>
@@ -3005,87 +3047,87 @@
     </row>
     <row r="30" spans="1:7" ht="81.95" customHeight="1">
       <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="2">
+        <v>1117</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="81.95" customHeight="1">
       <c r="A31">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="2">
-        <v>1117</v>
+        <v>5</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="81.95" customHeight="1">
       <c r="A32">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>5</v>
+        <v>14</v>
+      </c>
+      <c r="D32" s="2">
+        <v>1121</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="81.95" customHeight="1">
       <c r="A33">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="2">
-        <v>1121</v>
+        <v>5</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="81.95" customHeight="1">
       <c r="A34">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>5</v>
@@ -3105,7 +3147,7 @@
     </row>
     <row r="35" spans="1:7" ht="81.95" customHeight="1">
       <c r="A35">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>5</v>
@@ -3125,7 +3167,7 @@
     </row>
     <row r="36" spans="1:7" ht="81.95" customHeight="1">
       <c r="A36">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>5</v>
@@ -3145,19 +3187,19 @@
     </row>
     <row r="37" spans="1:7" ht="81.95" customHeight="1">
       <c r="A37">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>5</v>
+        <v>32</v>
+      </c>
+      <c r="D37" s="2">
+        <v>1076</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>5</v>
@@ -3165,7 +3207,7 @@
     </row>
     <row r="38" spans="1:7" ht="81.95" customHeight="1">
       <c r="A38">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>5</v>
@@ -3185,7 +3227,7 @@
     </row>
     <row r="39" spans="1:7" ht="81.95" customHeight="1">
       <c r="A39">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>5</v>
@@ -3205,19 +3247,19 @@
     </row>
     <row r="40" spans="1:7" ht="81.95" customHeight="1">
       <c r="A40">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D40" s="2">
-        <v>1076</v>
+        <v>5</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>5</v>
@@ -3225,7 +3267,7 @@
     </row>
     <row r="41" spans="1:7" ht="81.95" customHeight="1">
       <c r="A41">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>5</v>
@@ -3245,27 +3287,27 @@
     </row>
     <row r="42" spans="1:7" ht="81.95" customHeight="1">
       <c r="A42">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>5</v>
+        <v>16</v>
+      </c>
+      <c r="D42" s="2">
+        <v>1018</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="81.95" customHeight="1">
       <c r="A43">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>5</v>
@@ -3285,7 +3327,7 @@
     </row>
     <row r="44" spans="1:7" ht="81.95" customHeight="1">
       <c r="A44">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>5</v>
@@ -3305,27 +3347,27 @@
     </row>
     <row r="45" spans="1:7" ht="81.95" customHeight="1">
       <c r="A45">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D45" s="2">
-        <v>1018</v>
+        <v>5</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="81.95" customHeight="1">
       <c r="A46">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>5</v>
@@ -3345,101 +3387,41 @@
     </row>
     <row r="47" spans="1:7" ht="81.95" customHeight="1">
       <c r="A47">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="D47" s="2">
+        <v>1024</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="81.95" customHeight="1">
       <c r="A48">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
+      </c>
+      <c r="D48" s="2">
+        <v>1201</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="81.95" customHeight="1">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="81.95" customHeight="1">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D50" s="2">
-        <v>1024</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="81.95" customHeight="1">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D51" s="2">
-        <v>1201</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" s="2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>